<commit_message>
Atualiza diversos arquivos HTML para incluir links de navegação para a página inicial
</commit_message>
<xml_diff>
--- a/nao_positivados_06-2026.xlsx
+++ b/nao_positivados_06-2026.xlsx
@@ -36008,7 +36008,7 @@
         <v>6122</v>
       </c>
       <c r="D467" t="s">
-        <v>7468</v>
+        <v>7469</v>
       </c>
       <c r="E467" t="s">
         <v>8030</v>
@@ -36028,7 +36028,7 @@
         <v>6255</v>
       </c>
       <c r="D468" t="s">
-        <v>7469</v>
+        <v>7468</v>
       </c>
       <c r="E468" t="s">
         <v>8030</v>
@@ -93414,7 +93414,7 @@
         <v>6711</v>
       </c>
       <c r="D3112" t="s">
-        <v>7769</v>
+        <v>7426</v>
       </c>
       <c r="E3112" t="s">
         <v>8129</v>
@@ -93437,7 +93437,7 @@
         <v>6019</v>
       </c>
       <c r="D3113" t="s">
-        <v>7624</v>
+        <v>7625</v>
       </c>
       <c r="E3113" t="s">
         <v>8129</v>

</xml_diff>

<commit_message>
Refactor main pipeline: remove catalog export step, update WhatsApp alert step, and delete Catalogo page
</commit_message>
<xml_diff>
--- a/nao_positivados_06-2026.xlsx
+++ b/nao_positivados_06-2026.xlsx
@@ -22414,12 +22414,15 @@
     <t>APERITIVO APEROL 750 ML</t>
   </si>
   <si>
-    <t>VINHO TINTO QUINTA DE VENTOZELO SOUSAO</t>
+    <t>VINHO QUINTA DE VENTOZELO TINTO CÃ0</t>
   </si>
   <si>
     <t>HUMB. CANALE DENARIO MALBEC 750ML</t>
   </si>
   <si>
+    <t>VINHO LA TOGATA ROSSO 750ML</t>
+  </si>
+  <si>
     <t>VINHO LA TOGATA BRUNELLO ETQ AZUL 750ML</t>
   </si>
   <si>
@@ -22427,9 +22430,6 @@
   </si>
   <si>
     <t>VINHO BAROLO BUSSIA RISERVA 750ML</t>
-  </si>
-  <si>
-    <t>VINHO LA TOGATA ROSSO 750ML</t>
   </si>
   <si>
     <t>HUMB. CANALE DENARIO RESERVA CAB. FRANC</t>
@@ -35925,7 +35925,7 @@
         <v>6252</v>
       </c>
       <c r="D463" t="s">
-        <v>7468</v>
+        <v>7469</v>
       </c>
       <c r="E463" t="s">
         <v>8030</v>
@@ -35945,7 +35945,7 @@
         <v>6253</v>
       </c>
       <c r="D464" t="s">
-        <v>7469</v>
+        <v>7470</v>
       </c>
       <c r="E464" t="s">
         <v>8030</v>
@@ -35988,7 +35988,7 @@
         <v>6254</v>
       </c>
       <c r="D466" t="s">
-        <v>7470</v>
+        <v>7471</v>
       </c>
       <c r="E466" t="s">
         <v>8030</v>
@@ -36008,7 +36008,7 @@
         <v>6122</v>
       </c>
       <c r="D467" t="s">
-        <v>7471</v>
+        <v>7468</v>
       </c>
       <c r="E467" t="s">
         <v>8030</v>
@@ -36028,7 +36028,7 @@
         <v>6255</v>
       </c>
       <c r="D468" t="s">
-        <v>7468</v>
+        <v>7469</v>
       </c>
       <c r="E468" t="s">
         <v>8030</v>
@@ -36048,7 +36048,7 @@
         <v>6092</v>
       </c>
       <c r="D469" t="s">
-        <v>7471</v>
+        <v>7468</v>
       </c>
       <c r="E469" t="s">
         <v>8030</v>
@@ -36068,7 +36068,7 @@
         <v>6066</v>
       </c>
       <c r="D470" t="s">
-        <v>7468</v>
+        <v>7469</v>
       </c>
       <c r="E470" t="s">
         <v>8030</v>
@@ -62732,7 +62732,7 @@
         <v>6622</v>
       </c>
       <c r="D1679" t="s">
-        <v>7471</v>
+        <v>7468</v>
       </c>
       <c r="E1679" t="s">
         <v>8059</v>
@@ -64204,7 +64204,7 @@
         <v>6127</v>
       </c>
       <c r="D1743" t="s">
-        <v>7469</v>
+        <v>7470</v>
       </c>
       <c r="E1743" t="s">
         <v>8059</v>
@@ -93414,7 +93414,7 @@
         <v>6711</v>
       </c>
       <c r="D3112" t="s">
-        <v>7769</v>
+        <v>7426</v>
       </c>
       <c r="E3112" t="s">
         <v>8129</v>
@@ -93437,7 +93437,7 @@
         <v>6019</v>
       </c>
       <c r="D3113" t="s">
-        <v>7623</v>
+        <v>7624</v>
       </c>
       <c r="E3113" t="s">
         <v>8129</v>

</xml_diff>